<commit_message>
Updates for MaTrace Run
</commit_message>
<xml_diff>
--- a/docs/LL_IEooc_Methods3_Software1_Data.xlsx
+++ b/docs/LL_IEooc_Methods3_Software1_Data.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elanphear\Code\ODYM\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ABC267E-6C0F-4ED1-9E54-C5D189422440}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6348540A-5A3B-49E6-8E9F-5180779F517C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
     <sheet name="Data_Batteries_US" sheetId="2" r:id="rId2"/>
     <sheet name="Data_Batteries_US (2)" sheetId="3" r:id="rId3"/>
+    <sheet name="Data_Batteries_US (3)" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="10">
   <si>
     <t>Country:</t>
   </si>
@@ -62,6 +63,12 @@
   </si>
   <si>
     <t>Scenario for future battery stock, basic, kt</t>
+  </si>
+  <si>
+    <t>Stock diff year over year</t>
+  </si>
+  <si>
+    <t>J2 taken from code</t>
   </si>
 </sst>
 </file>
@@ -2716,7 +2723,7 @@
         <v>2025</v>
       </c>
       <c r="J3">
-        <v>1519.4404879999997</v>
+        <v>5609.5043013300001</v>
       </c>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.35">
@@ -2730,7 +2737,7 @@
         <v>2026</v>
       </c>
       <c r="J4">
-        <v>1962.2205919999997</v>
+        <v>6052.2844053299996</v>
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.35">
@@ -2744,7 +2751,7 @@
         <v>2027</v>
       </c>
       <c r="J5">
-        <v>2475.3879439999996</v>
+        <v>6565.45175733</v>
       </c>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.35">
@@ -2758,7 +2765,7 @@
         <v>2028</v>
       </c>
       <c r="J6">
-        <v>3148.5304129999995</v>
+        <v>7238.5942263300003</v>
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.35">
@@ -2772,7 +2779,7 @@
         <v>2029</v>
       </c>
       <c r="J7">
-        <v>4025.6357349999994</v>
+        <v>8115.6995483299997</v>
       </c>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.35">
@@ -2786,7 +2793,7 @@
         <v>2030</v>
       </c>
       <c r="J8">
-        <v>5116.2194139999992</v>
+        <v>9206.2832273299991</v>
       </c>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.35">
@@ -2800,7 +2807,7 @@
         <v>2031</v>
       </c>
       <c r="J9">
-        <v>5719.8720809999986</v>
+        <v>9809.9358943299994</v>
       </c>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.35">
@@ -2814,7 +2821,7 @@
         <v>2032</v>
       </c>
       <c r="J10">
-        <v>6409.7031809999989</v>
+        <v>10499.766994329999</v>
       </c>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.35">
@@ -2828,7 +2835,7 @@
         <v>2033</v>
       </c>
       <c r="J11">
-        <v>7140.9778219999989</v>
+        <v>11231.041635329999</v>
       </c>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.35">
@@ -2842,7 +2849,7 @@
         <v>2034</v>
       </c>
       <c r="J12">
-        <v>7948.4108469999983</v>
+        <v>12038.474660329997</v>
       </c>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.35">
@@ -2856,7 +2863,7 @@
         <v>2035</v>
       </c>
       <c r="J13">
-        <v>8845.9663439999986</v>
+        <v>12936.030157329998</v>
       </c>
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.35">
@@ -2870,7 +2877,7 @@
         <v>2036</v>
       </c>
       <c r="J14">
-        <v>9200</v>
+        <v>13290.06381333</v>
       </c>
     </row>
     <row r="15" spans="2:10" x14ac:dyDescent="0.35">
@@ -2884,7 +2891,7 @@
         <v>2037</v>
       </c>
       <c r="J15">
-        <v>9500</v>
+        <v>13590.06381333</v>
       </c>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.35">
@@ -2898,7 +2905,7 @@
         <v>2038</v>
       </c>
       <c r="J16">
-        <v>9700</v>
+        <v>13790.06381333</v>
       </c>
     </row>
     <row r="17" spans="3:10" x14ac:dyDescent="0.35">
@@ -2912,7 +2919,7 @@
         <v>2039</v>
       </c>
       <c r="J17">
-        <v>10000</v>
+        <v>14090.06381333</v>
       </c>
     </row>
     <row r="18" spans="3:10" x14ac:dyDescent="0.35">
@@ -2926,7 +2933,7 @@
         <v>2040</v>
       </c>
       <c r="J18">
-        <v>12000</v>
+        <v>16090.06381333</v>
       </c>
     </row>
     <row r="19" spans="3:10" x14ac:dyDescent="0.35">
@@ -2940,7 +2947,7 @@
         <v>2041</v>
       </c>
       <c r="J19">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="20" spans="3:10" x14ac:dyDescent="0.35">
@@ -2954,7 +2961,7 @@
         <v>2042</v>
       </c>
       <c r="J20">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="21" spans="3:10" x14ac:dyDescent="0.35">
@@ -2968,7 +2975,7 @@
         <v>2043</v>
       </c>
       <c r="J21">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="22" spans="3:10" x14ac:dyDescent="0.35">
@@ -2982,7 +2989,7 @@
         <v>2044</v>
       </c>
       <c r="J22">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="23" spans="3:10" x14ac:dyDescent="0.35">
@@ -2996,7 +3003,7 @@
         <v>2045</v>
       </c>
       <c r="J23">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="24" spans="3:10" x14ac:dyDescent="0.35">
@@ -3010,7 +3017,7 @@
         <v>2046</v>
       </c>
       <c r="J24">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="25" spans="3:10" x14ac:dyDescent="0.35">
@@ -3024,7 +3031,7 @@
         <v>2047</v>
       </c>
       <c r="J25">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="26" spans="3:10" x14ac:dyDescent="0.35">
@@ -3038,7 +3045,7 @@
         <v>2048</v>
       </c>
       <c r="J26">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="27" spans="3:10" x14ac:dyDescent="0.35">
@@ -3052,7 +3059,7 @@
         <v>2049</v>
       </c>
       <c r="J27">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="28" spans="3:10" x14ac:dyDescent="0.35">
@@ -3061,7 +3068,7 @@
         <v>2050</v>
       </c>
       <c r="J28">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="29" spans="3:10" x14ac:dyDescent="0.35">
@@ -3070,7 +3077,7 @@
         <v>2051</v>
       </c>
       <c r="J29">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="30" spans="3:10" x14ac:dyDescent="0.35">
@@ -3079,7 +3086,7 @@
         <v>2052</v>
       </c>
       <c r="J30">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="31" spans="3:10" x14ac:dyDescent="0.35">
@@ -3088,7 +3095,7 @@
         <v>2053</v>
       </c>
       <c r="J31">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="32" spans="3:10" x14ac:dyDescent="0.35">
@@ -3097,7 +3104,7 @@
         <v>2054</v>
       </c>
       <c r="J32">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="33" spans="3:10" x14ac:dyDescent="0.35">
@@ -3106,7 +3113,7 @@
         <v>2055</v>
       </c>
       <c r="J33">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="34" spans="3:10" x14ac:dyDescent="0.35">
@@ -3115,7 +3122,7 @@
         <v>2056</v>
       </c>
       <c r="J34">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="35" spans="3:10" x14ac:dyDescent="0.35">
@@ -3124,7 +3131,7 @@
         <v>2057</v>
       </c>
       <c r="J35">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="36" spans="3:10" x14ac:dyDescent="0.35">
@@ -3133,7 +3140,7 @@
         <v>2058</v>
       </c>
       <c r="J36">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="37" spans="3:10" x14ac:dyDescent="0.35">
@@ -3142,7 +3149,7 @@
         <v>2059</v>
       </c>
       <c r="J37">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="38" spans="3:10" x14ac:dyDescent="0.35">
@@ -3151,7 +3158,7 @@
         <v>2060</v>
       </c>
       <c r="J38">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="39" spans="3:10" x14ac:dyDescent="0.35">
@@ -3160,7 +3167,7 @@
         <v>2061</v>
       </c>
       <c r="J39">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="40" spans="3:10" x14ac:dyDescent="0.35">
@@ -3169,7 +3176,7 @@
         <v>2062</v>
       </c>
       <c r="J40">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="41" spans="3:10" x14ac:dyDescent="0.35">
@@ -3178,7 +3185,7 @@
         <v>2063</v>
       </c>
       <c r="J41">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="42" spans="3:10" x14ac:dyDescent="0.35">
@@ -3187,7 +3194,7 @@
         <v>2064</v>
       </c>
       <c r="J42">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="43" spans="3:10" x14ac:dyDescent="0.35">
@@ -3196,7 +3203,7 @@
         <v>2065</v>
       </c>
       <c r="J43">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="44" spans="3:10" x14ac:dyDescent="0.35">
@@ -3205,7 +3212,7 @@
         <v>2066</v>
       </c>
       <c r="J44">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="45" spans="3:10" x14ac:dyDescent="0.35">
@@ -3214,7 +3221,7 @@
         <v>2067</v>
       </c>
       <c r="J45">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="46" spans="3:10" x14ac:dyDescent="0.35">
@@ -3223,7 +3230,7 @@
         <v>2068</v>
       </c>
       <c r="J46">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="47" spans="3:10" x14ac:dyDescent="0.35">
@@ -3232,7 +3239,7 @@
         <v>2069</v>
       </c>
       <c r="J47">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="48" spans="3:10" x14ac:dyDescent="0.35">
@@ -3241,7 +3248,7 @@
         <v>2070</v>
       </c>
       <c r="J48">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="49" spans="3:10" x14ac:dyDescent="0.35">
@@ -3250,7 +3257,7 @@
         <v>2071</v>
       </c>
       <c r="J49">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="50" spans="3:10" x14ac:dyDescent="0.35">
@@ -3259,7 +3266,7 @@
         <v>2072</v>
       </c>
       <c r="J50">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="51" spans="3:10" x14ac:dyDescent="0.35">
@@ -3268,7 +3275,7 @@
         <v>2073</v>
       </c>
       <c r="J51">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="52" spans="3:10" x14ac:dyDescent="0.35">
@@ -3277,7 +3284,7 @@
         <v>2074</v>
       </c>
       <c r="J52">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="53" spans="3:10" x14ac:dyDescent="0.35">
@@ -3286,7 +3293,7 @@
         <v>2075</v>
       </c>
       <c r="J53">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="54" spans="3:10" x14ac:dyDescent="0.35">
@@ -3295,7 +3302,7 @@
         <v>2076</v>
       </c>
       <c r="J54">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="55" spans="3:10" x14ac:dyDescent="0.35">
@@ -3304,7 +3311,7 @@
         <v>2077</v>
       </c>
       <c r="J55">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="56" spans="3:10" x14ac:dyDescent="0.35">
@@ -3313,7 +3320,7 @@
         <v>2078</v>
       </c>
       <c r="J56">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="57" spans="3:10" x14ac:dyDescent="0.35">
@@ -3322,7 +3329,7 @@
         <v>2079</v>
       </c>
       <c r="J57">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="58" spans="3:10" x14ac:dyDescent="0.35">
@@ -3331,7 +3338,7 @@
         <v>2080</v>
       </c>
       <c r="J58">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="59" spans="3:10" x14ac:dyDescent="0.35">
@@ -3340,7 +3347,7 @@
         <v>2081</v>
       </c>
       <c r="J59">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="60" spans="3:10" x14ac:dyDescent="0.35">
@@ -3349,7 +3356,7 @@
         <v>2082</v>
       </c>
       <c r="J60">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="61" spans="3:10" x14ac:dyDescent="0.35">
@@ -3358,7 +3365,7 @@
         <v>2083</v>
       </c>
       <c r="J61">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="62" spans="3:10" x14ac:dyDescent="0.35">
@@ -3367,7 +3374,7 @@
         <v>2084</v>
       </c>
       <c r="J62">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="63" spans="3:10" x14ac:dyDescent="0.35">
@@ -3376,7 +3383,7 @@
         <v>2085</v>
       </c>
       <c r="J63">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="64" spans="3:10" x14ac:dyDescent="0.35">
@@ -3385,7 +3392,7 @@
         <v>2086</v>
       </c>
       <c r="J64">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="65" spans="3:10" x14ac:dyDescent="0.35">
@@ -3394,7 +3401,7 @@
         <v>2087</v>
       </c>
       <c r="J65">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="66" spans="3:10" x14ac:dyDescent="0.35">
@@ -3403,7 +3410,7 @@
         <v>2088</v>
       </c>
       <c r="J66">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="67" spans="3:10" x14ac:dyDescent="0.35">
@@ -3412,7 +3419,7 @@
         <v>2089</v>
       </c>
       <c r="J67">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="68" spans="3:10" x14ac:dyDescent="0.35">
@@ -3421,7 +3428,7 @@
         <v>2090</v>
       </c>
       <c r="J68">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="69" spans="3:10" x14ac:dyDescent="0.35">
@@ -3430,7 +3437,7 @@
         <v>2091</v>
       </c>
       <c r="J69">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="70" spans="3:10" x14ac:dyDescent="0.35">
@@ -3439,7 +3446,7 @@
         <v>2092</v>
       </c>
       <c r="J70">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="71" spans="3:10" x14ac:dyDescent="0.35">
@@ -3448,7 +3455,7 @@
         <v>2093</v>
       </c>
       <c r="J71">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="72" spans="3:10" x14ac:dyDescent="0.35">
@@ -3457,7 +3464,7 @@
         <v>2094</v>
       </c>
       <c r="J72">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="73" spans="3:10" x14ac:dyDescent="0.35">
@@ -3466,7 +3473,7 @@
         <v>2095</v>
       </c>
       <c r="J73">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="74" spans="3:10" x14ac:dyDescent="0.35">
@@ -3475,7 +3482,7 @@
         <v>2096</v>
       </c>
       <c r="J74">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="75" spans="3:10" x14ac:dyDescent="0.35">
@@ -3484,7 +3491,7 @@
         <v>2097</v>
       </c>
       <c r="J75">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="76" spans="3:10" x14ac:dyDescent="0.35">
@@ -3493,7 +3500,7 @@
         <v>2098</v>
       </c>
       <c r="J76">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="77" spans="3:10" x14ac:dyDescent="0.35">
@@ -3502,7 +3509,7 @@
         <v>2099</v>
       </c>
       <c r="J77">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="78" spans="3:10" x14ac:dyDescent="0.35">
@@ -3511,7 +3518,7 @@
         <v>2100</v>
       </c>
       <c r="J78">
-        <v>13000</v>
+        <v>17090.063813330002</v>
       </c>
     </row>
     <row r="79" spans="3:10" x14ac:dyDescent="0.35">
@@ -5383,4 +5390,1236 @@
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{115570CE-A599-420B-9BD7-E20CBAF8501B}">
+  <dimension ref="B1:L103"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="3" max="3" width="21.81640625" customWidth="1"/>
+    <col min="4" max="4" width="17.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B2" s="1"/>
+      <c r="D2" s="3"/>
+      <c r="I2" s="1">
+        <v>2024</v>
+      </c>
+      <c r="J2">
+        <v>5226.1918033299999</v>
+      </c>
+      <c r="K2" t="s">
+        <v>8</v>
+      </c>
+      <c r="L2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="1">
+        <v>2000</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="I3" s="1">
+        <v>2025</v>
+      </c>
+      <c r="J3">
+        <f>J2+K3</f>
+        <v>5609.5043013300001</v>
+      </c>
+      <c r="K3">
+        <v>383.31249800000001</v>
+      </c>
+    </row>
+    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="C4" s="1">
+        <v>2001</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="I4" s="1">
+        <v>2026</v>
+      </c>
+      <c r="J4">
+        <f t="shared" ref="J4:J67" si="0">J3+K4</f>
+        <v>6052.2844053299996</v>
+      </c>
+      <c r="K4">
+        <v>442.78010399999994</v>
+      </c>
+    </row>
+    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="C5" s="1">
+        <v>2002</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="I5" s="1">
+        <v>2027</v>
+      </c>
+      <c r="J5">
+        <f t="shared" si="0"/>
+        <v>6565.45175733</v>
+      </c>
+      <c r="K5">
+        <v>513.16735199999994</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="C6" s="1">
+        <v>2003</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="I6" s="1">
+        <v>2028</v>
+      </c>
+      <c r="J6">
+        <f t="shared" si="0"/>
+        <v>7238.5942263300003</v>
+      </c>
+      <c r="K6">
+        <v>673.14246899999989</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="C7" s="1">
+        <v>2004</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="I7" s="1">
+        <v>2029</v>
+      </c>
+      <c r="J7">
+        <f t="shared" si="0"/>
+        <v>8115.6995483299997</v>
+      </c>
+      <c r="K7">
+        <v>877.10532199999989</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="C8" s="1">
+        <v>2005</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="I8" s="1">
+        <v>2030</v>
+      </c>
+      <c r="J8">
+        <f t="shared" si="0"/>
+        <v>9206.2832273299991</v>
+      </c>
+      <c r="K8">
+        <v>1090.5836789999998</v>
+      </c>
+    </row>
+    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="C9" s="1">
+        <v>2006</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="I9" s="1">
+        <v>2031</v>
+      </c>
+      <c r="J9">
+        <f t="shared" si="0"/>
+        <v>9809.9358943299994</v>
+      </c>
+      <c r="K9">
+        <v>603.65266699999938</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="C10" s="1">
+        <v>2007</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="I10" s="1">
+        <v>2032</v>
+      </c>
+      <c r="J10">
+        <f t="shared" si="0"/>
+        <v>10499.766994329999</v>
+      </c>
+      <c r="K10">
+        <v>689.83110000000033</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="C11" s="1">
+        <v>2008</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="I11" s="1">
+        <v>2033</v>
+      </c>
+      <c r="J11">
+        <f t="shared" si="0"/>
+        <v>11231.041635329999</v>
+      </c>
+      <c r="K11">
+        <v>731.27464099999997</v>
+      </c>
+    </row>
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="C12" s="1">
+        <v>2009</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="I12" s="1">
+        <v>2034</v>
+      </c>
+      <c r="J12">
+        <f t="shared" si="0"/>
+        <v>12038.474660329997</v>
+      </c>
+      <c r="K12">
+        <v>807.43302499999936</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="C13" s="1">
+        <v>2010</v>
+      </c>
+      <c r="D13">
+        <v>20</v>
+      </c>
+      <c r="I13" s="1">
+        <v>2035</v>
+      </c>
+      <c r="J13">
+        <f t="shared" si="0"/>
+        <v>12936.030157329998</v>
+      </c>
+      <c r="K13">
+        <v>897.55549700000029</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="C14" s="1">
+        <v>2011</v>
+      </c>
+      <c r="D14">
+        <v>35</v>
+      </c>
+      <c r="I14" s="1">
+        <v>2036</v>
+      </c>
+      <c r="J14">
+        <f t="shared" si="0"/>
+        <v>13290.06381333</v>
+      </c>
+      <c r="K14">
+        <v>354.03365600000143</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="C15" s="1">
+        <v>2012</v>
+      </c>
+      <c r="D15">
+        <v>80</v>
+      </c>
+      <c r="I15" s="1">
+        <v>2037</v>
+      </c>
+      <c r="J15">
+        <f t="shared" si="0"/>
+        <v>13590.06381333</v>
+      </c>
+      <c r="K15">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="C16" s="1">
+        <v>2013</v>
+      </c>
+      <c r="D16">
+        <v>150</v>
+      </c>
+      <c r="I16" s="1">
+        <v>2038</v>
+      </c>
+      <c r="J16">
+        <f t="shared" si="0"/>
+        <v>13790.06381333</v>
+      </c>
+      <c r="K16">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="17" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C17" s="1">
+        <v>2014</v>
+      </c>
+      <c r="D17">
+        <v>257.01736999999997</v>
+      </c>
+      <c r="I17" s="1">
+        <v>2039</v>
+      </c>
+      <c r="J17">
+        <f t="shared" si="0"/>
+        <v>14090.06381333</v>
+      </c>
+      <c r="K17">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="18" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C18" s="1">
+        <v>2015</v>
+      </c>
+      <c r="D18">
+        <v>280</v>
+      </c>
+      <c r="I18" s="1">
+        <v>2040</v>
+      </c>
+      <c r="J18">
+        <f t="shared" si="0"/>
+        <v>16090.06381333</v>
+      </c>
+      <c r="K18">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="19" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C19" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D19">
+        <v>309.16799999999995</v>
+      </c>
+      <c r="I19" s="1">
+        <v>2041</v>
+      </c>
+      <c r="J19">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K19">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="20" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C20" s="1">
+        <v>2017</v>
+      </c>
+      <c r="D20">
+        <v>350</v>
+      </c>
+      <c r="I20" s="1">
+        <v>2042</v>
+      </c>
+      <c r="J20">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C21" s="1">
+        <v>2018</v>
+      </c>
+      <c r="D21">
+        <v>400</v>
+      </c>
+      <c r="I21" s="1">
+        <v>2043</v>
+      </c>
+      <c r="J21">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C22" s="1">
+        <v>2019</v>
+      </c>
+      <c r="D22">
+        <v>490</v>
+      </c>
+      <c r="I22" s="1">
+        <v>2044</v>
+      </c>
+      <c r="J22">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C23" s="1">
+        <v>2020</v>
+      </c>
+      <c r="D23">
+        <v>530</v>
+      </c>
+      <c r="I23" s="1">
+        <v>2045</v>
+      </c>
+      <c r="J23">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C24" s="1">
+        <v>2021</v>
+      </c>
+      <c r="D24">
+        <v>720</v>
+      </c>
+      <c r="I24" s="1">
+        <v>2046</v>
+      </c>
+      <c r="J24">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C25" s="1">
+        <v>2022</v>
+      </c>
+      <c r="D25">
+        <v>800</v>
+      </c>
+      <c r="I25" s="1">
+        <v>2047</v>
+      </c>
+      <c r="J25">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C26" s="1">
+        <v>2023</v>
+      </c>
+      <c r="D26">
+        <v>928.57749999999987</v>
+      </c>
+      <c r="I26" s="1">
+        <v>2048</v>
+      </c>
+      <c r="J26">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C27" s="1">
+        <v>2024</v>
+      </c>
+      <c r="D27">
+        <v>1136.1279899999997</v>
+      </c>
+      <c r="I27" s="1">
+        <v>2049</v>
+      </c>
+      <c r="J27">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C28" s="1"/>
+      <c r="I28" s="1">
+        <v>2050</v>
+      </c>
+      <c r="J28">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C29" s="1"/>
+      <c r="I29" s="1">
+        <v>2051</v>
+      </c>
+      <c r="J29">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C30" s="1"/>
+      <c r="I30" s="1">
+        <v>2052</v>
+      </c>
+      <c r="J30">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C31" s="1"/>
+      <c r="I31" s="1">
+        <v>2053</v>
+      </c>
+      <c r="J31">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C32" s="1"/>
+      <c r="I32" s="1">
+        <v>2054</v>
+      </c>
+      <c r="J32">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C33" s="1"/>
+      <c r="I33" s="1">
+        <v>2055</v>
+      </c>
+      <c r="J33">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C34" s="1"/>
+      <c r="I34" s="1">
+        <v>2056</v>
+      </c>
+      <c r="J34">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C35" s="1"/>
+      <c r="I35" s="1">
+        <v>2057</v>
+      </c>
+      <c r="J35">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C36" s="1"/>
+      <c r="I36" s="1">
+        <v>2058</v>
+      </c>
+      <c r="J36">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C37" s="1"/>
+      <c r="I37" s="1">
+        <v>2059</v>
+      </c>
+      <c r="J37">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C38" s="1"/>
+      <c r="I38" s="1">
+        <v>2060</v>
+      </c>
+      <c r="J38">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C39" s="1"/>
+      <c r="I39" s="1">
+        <v>2061</v>
+      </c>
+      <c r="J39">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C40" s="1"/>
+      <c r="I40" s="1">
+        <v>2062</v>
+      </c>
+      <c r="J40">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C41" s="1"/>
+      <c r="I41" s="1">
+        <v>2063</v>
+      </c>
+      <c r="J41">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C42" s="1"/>
+      <c r="I42" s="1">
+        <v>2064</v>
+      </c>
+      <c r="J42">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C43" s="1"/>
+      <c r="I43" s="1">
+        <v>2065</v>
+      </c>
+      <c r="J43">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C44" s="1"/>
+      <c r="I44" s="1">
+        <v>2066</v>
+      </c>
+      <c r="J44">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C45" s="1"/>
+      <c r="I45" s="1">
+        <v>2067</v>
+      </c>
+      <c r="J45">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C46" s="1"/>
+      <c r="I46" s="1">
+        <v>2068</v>
+      </c>
+      <c r="J46">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C47" s="1"/>
+      <c r="I47" s="1">
+        <v>2069</v>
+      </c>
+      <c r="J47">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C48" s="1"/>
+      <c r="I48" s="1">
+        <v>2070</v>
+      </c>
+      <c r="J48">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K48">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C49" s="1"/>
+      <c r="I49" s="1">
+        <v>2071</v>
+      </c>
+      <c r="J49">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C50" s="1"/>
+      <c r="I50" s="1">
+        <v>2072</v>
+      </c>
+      <c r="J50">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C51" s="1"/>
+      <c r="I51" s="1">
+        <v>2073</v>
+      </c>
+      <c r="J51">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K51">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C52" s="1"/>
+      <c r="I52" s="1">
+        <v>2074</v>
+      </c>
+      <c r="J52">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K52">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C53" s="1"/>
+      <c r="I53" s="1">
+        <v>2075</v>
+      </c>
+      <c r="J53">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C54" s="1"/>
+      <c r="I54" s="1">
+        <v>2076</v>
+      </c>
+      <c r="J54">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K54">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C55" s="1"/>
+      <c r="I55" s="1">
+        <v>2077</v>
+      </c>
+      <c r="J55">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K55">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C56" s="1"/>
+      <c r="I56" s="1">
+        <v>2078</v>
+      </c>
+      <c r="J56">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K56">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C57" s="1"/>
+      <c r="I57" s="1">
+        <v>2079</v>
+      </c>
+      <c r="J57">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K57">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C58" s="1"/>
+      <c r="I58" s="1">
+        <v>2080</v>
+      </c>
+      <c r="J58">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C59" s="1"/>
+      <c r="I59" s="1">
+        <v>2081</v>
+      </c>
+      <c r="J59">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K59">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C60" s="1"/>
+      <c r="I60" s="1">
+        <v>2082</v>
+      </c>
+      <c r="J60">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K60">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C61" s="1"/>
+      <c r="I61" s="1">
+        <v>2083</v>
+      </c>
+      <c r="J61">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K61">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C62" s="1"/>
+      <c r="I62" s="1">
+        <v>2084</v>
+      </c>
+      <c r="J62">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K62">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C63" s="1"/>
+      <c r="I63" s="1">
+        <v>2085</v>
+      </c>
+      <c r="J63">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K63">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C64" s="1"/>
+      <c r="I64" s="1">
+        <v>2086</v>
+      </c>
+      <c r="J64">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K64">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C65" s="1"/>
+      <c r="I65" s="1">
+        <v>2087</v>
+      </c>
+      <c r="J65">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K65">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C66" s="1"/>
+      <c r="I66" s="1">
+        <v>2088</v>
+      </c>
+      <c r="J66">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K66">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C67" s="1"/>
+      <c r="I67" s="1">
+        <v>2089</v>
+      </c>
+      <c r="J67">
+        <f t="shared" si="0"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K67">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C68" s="1"/>
+      <c r="I68" s="1">
+        <v>2090</v>
+      </c>
+      <c r="J68">
+        <f t="shared" ref="J68:J78" si="1">J67+K68</f>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K68">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C69" s="1"/>
+      <c r="I69" s="1">
+        <v>2091</v>
+      </c>
+      <c r="J69">
+        <f t="shared" si="1"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K69">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C70" s="1"/>
+      <c r="I70" s="1">
+        <v>2092</v>
+      </c>
+      <c r="J70">
+        <f t="shared" si="1"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C71" s="1"/>
+      <c r="I71" s="1">
+        <v>2093</v>
+      </c>
+      <c r="J71">
+        <f t="shared" si="1"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K71">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C72" s="1"/>
+      <c r="I72" s="1">
+        <v>2094</v>
+      </c>
+      <c r="J72">
+        <f t="shared" si="1"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K72">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C73" s="1"/>
+      <c r="I73" s="1">
+        <v>2095</v>
+      </c>
+      <c r="J73">
+        <f t="shared" si="1"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K73">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C74" s="1"/>
+      <c r="I74" s="1">
+        <v>2096</v>
+      </c>
+      <c r="J74">
+        <f t="shared" si="1"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K74">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C75" s="1"/>
+      <c r="I75" s="1">
+        <v>2097</v>
+      </c>
+      <c r="J75">
+        <f t="shared" si="1"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C76" s="1"/>
+      <c r="I76" s="1">
+        <v>2098</v>
+      </c>
+      <c r="J76">
+        <f t="shared" si="1"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K76">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C77" s="1"/>
+      <c r="I77" s="1">
+        <v>2099</v>
+      </c>
+      <c r="J77">
+        <f t="shared" si="1"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K77">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C78" s="1"/>
+      <c r="I78" s="1">
+        <v>2100</v>
+      </c>
+      <c r="J78">
+        <f t="shared" si="1"/>
+        <v>17090.063813330002</v>
+      </c>
+      <c r="K78">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C79" s="1"/>
+    </row>
+    <row r="80" spans="3:11" x14ac:dyDescent="0.35">
+      <c r="C80" s="1"/>
+    </row>
+    <row r="81" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C81" s="1"/>
+    </row>
+    <row r="82" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C82" s="1"/>
+    </row>
+    <row r="83" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C83" s="1"/>
+    </row>
+    <row r="84" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C84" s="1"/>
+    </row>
+    <row r="85" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C85" s="1"/>
+    </row>
+    <row r="86" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C86" s="1"/>
+    </row>
+    <row r="87" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C87" s="1"/>
+    </row>
+    <row r="88" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C88" s="1"/>
+    </row>
+    <row r="89" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C89" s="1"/>
+    </row>
+    <row r="90" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C90" s="1"/>
+    </row>
+    <row r="91" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C91" s="1"/>
+    </row>
+    <row r="92" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C92" s="1"/>
+    </row>
+    <row r="93" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C93" s="1"/>
+    </row>
+    <row r="94" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C94" s="1"/>
+    </row>
+    <row r="95" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C95" s="1"/>
+    </row>
+    <row r="96" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C96" s="1"/>
+    </row>
+    <row r="97" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C97" s="1"/>
+    </row>
+    <row r="98" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C98" s="1"/>
+    </row>
+    <row r="99" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C99" s="1"/>
+    </row>
+    <row r="100" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C100" s="1"/>
+    </row>
+    <row r="101" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C101" s="1"/>
+    </row>
+    <row r="102" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C102" s="1"/>
+    </row>
+    <row r="103" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C103" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>